<commit_message>
v1.0 2 june 2026 - FINAL
</commit_message>
<xml_diff>
--- a/peritonitis-prediction/PredictCRRTforKids_Database.xlsx
+++ b/peritonitis-prediction/PredictCRRTforKids_Database.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,176 +417,176 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH163"/>
+  <dimension ref="A1:AH164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Patient_ID</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>sex</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>vis</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ventilator</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>crrt</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>fo_at_crrt</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>lactic</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>platelet</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>sepsis</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>rsd</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>kreatinin</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>psofa</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>sodium</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>tls</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>age</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>prism_score</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>picu_stay</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>admss</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>fo</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>ph</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>hb</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>urine_v</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>alf</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>albumin</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>pelod</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>bicarbonate</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>potassium</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>hyperammonemia</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>survival probability</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
@@ -606,7 +594,7 @@
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="1" t="n">
         <v>45676</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -654,7 +642,7 @@
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="1" t="n">
         <v>45677</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -734,7 +722,7 @@
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="1" t="n">
         <v>45677</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -822,7 +810,7 @@
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="1" t="n">
         <v>45677</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -906,7 +894,7 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="1" t="n">
         <v>45677</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -1000,7 +988,7 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="1" t="n">
         <v>45677</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -1070,7 +1058,7 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="1" t="n">
         <v>45680</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -1174,7 +1162,7 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="1" t="n">
         <v>45680</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -1278,7 +1266,7 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="1" t="n">
         <v>45772</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -1352,7 +1340,7 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="1" t="n">
         <v>45777</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -1428,7 +1416,7 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -1544,7 +1532,7 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="1" t="n">
         <v>45843</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -1614,7 +1602,7 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="1" t="n">
         <v>45847</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -1688,7 +1676,7 @@
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="1" t="n">
         <v>45847</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -1760,7 +1748,7 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" s="2" t="n">
+      <c r="B16" s="1" t="n">
         <v>45847</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -1844,7 +1832,7 @@
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="1" t="n">
         <v>45847</v>
       </c>
       <c r="C17" t="inlineStr">
@@ -1912,7 +1900,7 @@
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" s="2" t="n">
+      <c r="B18" s="1" t="n">
         <v>45847</v>
       </c>
       <c r="C18" t="inlineStr">
@@ -2004,7 +1992,7 @@
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" s="2" t="n">
+      <c r="B19" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C19" t="inlineStr">
@@ -2090,7 +2078,7 @@
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C20" t="inlineStr">
@@ -2164,7 +2152,7 @@
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" s="2" t="n">
+      <c r="B21" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C21" t="inlineStr">
@@ -2238,7 +2226,7 @@
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" s="2" t="n">
+      <c r="B22" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C22" t="inlineStr">
@@ -2318,7 +2306,7 @@
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" s="2" t="n">
+      <c r="B23" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -2392,7 +2380,7 @@
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" s="2" t="n">
+      <c r="B24" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C24" t="inlineStr">
@@ -2464,7 +2452,7 @@
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
-      <c r="B25" s="2" t="n">
+      <c r="B25" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C25" t="inlineStr">
@@ -2540,7 +2528,7 @@
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
-      <c r="B26" s="2" t="n">
+      <c r="B26" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C26" t="inlineStr">
@@ -2630,7 +2618,7 @@
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
-      <c r="B27" s="2" t="n">
+      <c r="B27" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C27" t="inlineStr">
@@ -2720,7 +2708,7 @@
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
-      <c r="B28" s="2" t="n">
+      <c r="B28" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C28" t="inlineStr">
@@ -2800,7 +2788,7 @@
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
-      <c r="B29" s="2" t="n">
+      <c r="B29" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C29" t="inlineStr">
@@ -2886,7 +2874,7 @@
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
-      <c r="B30" s="2" t="n">
+      <c r="B30" s="1" t="n">
         <v>45848</v>
       </c>
       <c r="C30" t="inlineStr">
@@ -2980,7 +2968,7 @@
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
-      <c r="B31" s="2" t="n">
+      <c r="B31" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C31" t="inlineStr">
@@ -3070,7 +3058,7 @@
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
-      <c r="B32" s="2" t="n">
+      <c r="B32" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C32" t="inlineStr">
@@ -3156,7 +3144,7 @@
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
-      <c r="B33" s="2" t="n">
+      <c r="B33" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C33" t="inlineStr">
@@ -3240,7 +3228,7 @@
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
-      <c r="B34" s="2" t="n">
+      <c r="B34" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C34" t="inlineStr">
@@ -3330,7 +3318,7 @@
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
-      <c r="B35" s="2" t="n">
+      <c r="B35" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C35" t="inlineStr">
@@ -3420,7 +3408,7 @@
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
-      <c r="B36" s="2" t="n">
+      <c r="B36" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C36" t="inlineStr">
@@ -3510,7 +3498,7 @@
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
-      <c r="B37" s="2" t="n">
+      <c r="B37" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C37" t="inlineStr">
@@ -3602,7 +3590,7 @@
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
-      <c r="B38" s="2" t="n">
+      <c r="B38" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C38" t="inlineStr">
@@ -3692,7 +3680,7 @@
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
-      <c r="B39" s="2" t="n">
+      <c r="B39" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C39" t="inlineStr">
@@ -3782,7 +3770,7 @@
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
-      <c r="B40" s="2" t="n">
+      <c r="B40" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C40" t="inlineStr">
@@ -3872,7 +3860,7 @@
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
-      <c r="B41" s="2" t="n">
+      <c r="B41" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C41" t="inlineStr">
@@ -3964,7 +3952,7 @@
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
-      <c r="B42" s="2" t="n">
+      <c r="B42" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C42" t="inlineStr">
@@ -4052,7 +4040,7 @@
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
-      <c r="B43" s="2" t="n">
+      <c r="B43" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C43" t="inlineStr">
@@ -4140,7 +4128,7 @@
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
-      <c r="B44" s="2" t="n">
+      <c r="B44" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C44" t="inlineStr">
@@ -4240,7 +4228,7 @@
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
-      <c r="B45" s="2" t="n">
+      <c r="B45" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C45" t="inlineStr">
@@ -4334,7 +4322,7 @@
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
-      <c r="B46" s="2" t="n">
+      <c r="B46" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C46" t="inlineStr">
@@ -4434,7 +4422,7 @@
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
-      <c r="B47" s="2" t="n">
+      <c r="B47" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C47" t="inlineStr">
@@ -4532,7 +4520,7 @@
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
-      <c r="B48" s="2" t="n">
+      <c r="B48" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C48" t="inlineStr">
@@ -4616,7 +4604,7 @@
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
-      <c r="B49" s="2" t="n">
+      <c r="B49" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C49" t="inlineStr">
@@ -4690,7 +4678,7 @@
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
-      <c r="B50" s="2" t="n">
+      <c r="B50" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C50" t="inlineStr">
@@ -4780,7 +4768,7 @@
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
-      <c r="B51" s="2" t="n">
+      <c r="B51" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C51" t="inlineStr">
@@ -4870,7 +4858,7 @@
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
-      <c r="B52" s="2" t="n">
+      <c r="B52" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C52" t="inlineStr">
@@ -4962,7 +4950,7 @@
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
-      <c r="B53" s="2" t="n">
+      <c r="B53" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C53" t="inlineStr">
@@ -5056,7 +5044,7 @@
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
-      <c r="B54" s="2" t="n">
+      <c r="B54" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C54" t="inlineStr">
@@ -5152,7 +5140,7 @@
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
-      <c r="B55" s="2" t="n">
+      <c r="B55" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C55" t="inlineStr">
@@ -5250,7 +5238,7 @@
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
-      <c r="B56" s="2" t="n">
+      <c r="B56" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C56" t="inlineStr">
@@ -5344,7 +5332,7 @@
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
-      <c r="B57" s="2" t="n">
+      <c r="B57" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C57" t="inlineStr">
@@ -5434,7 +5422,7 @@
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
-      <c r="B58" s="2" t="n">
+      <c r="B58" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C58" t="inlineStr">
@@ -5524,7 +5512,7 @@
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
-      <c r="B59" s="2" t="n">
+      <c r="B59" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C59" t="inlineStr">
@@ -5604,7 +5592,7 @@
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
-      <c r="B60" s="2" t="n">
+      <c r="B60" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C60" t="inlineStr">
@@ -5686,7 +5674,7 @@
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
-      <c r="B61" s="2" t="n">
+      <c r="B61" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C61" t="inlineStr">
@@ -5778,7 +5766,7 @@
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
-      <c r="B62" s="2" t="n">
+      <c r="B62" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C62" t="inlineStr">
@@ -5880,7 +5868,7 @@
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
-      <c r="B63" s="2" t="n">
+      <c r="B63" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C63" t="inlineStr">
@@ -5974,7 +5962,7 @@
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
-      <c r="B64" s="2" t="n">
+      <c r="B64" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C64" t="inlineStr">
@@ -6070,7 +6058,7 @@
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
-      <c r="B65" s="2" t="n">
+      <c r="B65" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C65" t="inlineStr">
@@ -6164,7 +6152,7 @@
     </row>
     <row r="66">
       <c r="A66" t="inlineStr"/>
-      <c r="B66" s="2" t="n">
+      <c r="B66" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C66" t="inlineStr">
@@ -6254,7 +6242,7 @@
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
-      <c r="B67" s="2" t="n">
+      <c r="B67" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C67" t="inlineStr">
@@ -6348,7 +6336,7 @@
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
-      <c r="B68" s="2" t="n">
+      <c r="B68" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C68" t="inlineStr">
@@ -6440,7 +6428,7 @@
     </row>
     <row r="69">
       <c r="A69" t="inlineStr"/>
-      <c r="B69" s="2" t="n">
+      <c r="B69" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C69" t="inlineStr">
@@ -6534,7 +6522,7 @@
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
-      <c r="B70" s="2" t="n">
+      <c r="B70" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C70" t="inlineStr">
@@ -6630,7 +6618,7 @@
     </row>
     <row r="71">
       <c r="A71" t="inlineStr"/>
-      <c r="B71" s="2" t="n">
+      <c r="B71" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C71" t="inlineStr">
@@ -6724,7 +6712,7 @@
     </row>
     <row r="72">
       <c r="A72" t="inlineStr"/>
-      <c r="B72" s="2" t="n">
+      <c r="B72" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C72" t="inlineStr">
@@ -6818,7 +6806,7 @@
     </row>
     <row r="73">
       <c r="A73" t="inlineStr"/>
-      <c r="B73" s="2" t="n">
+      <c r="B73" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C73" t="inlineStr">
@@ -6908,7 +6896,7 @@
     </row>
     <row r="74">
       <c r="A74" t="inlineStr"/>
-      <c r="B74" s="2" t="n">
+      <c r="B74" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C74" t="inlineStr">
@@ -6998,7 +6986,7 @@
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
-      <c r="B75" s="2" t="n">
+      <c r="B75" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C75" t="inlineStr">
@@ -7088,7 +7076,7 @@
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
-      <c r="B76" s="2" t="n">
+      <c r="B76" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C76" t="inlineStr">
@@ -7182,7 +7170,7 @@
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
-      <c r="B77" s="2" t="n">
+      <c r="B77" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C77" t="inlineStr">
@@ -7270,7 +7258,7 @@
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
-      <c r="B78" s="2" t="n">
+      <c r="B78" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C78" t="inlineStr">
@@ -7366,7 +7354,7 @@
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
-      <c r="B79" s="2" t="n">
+      <c r="B79" s="1" t="n">
         <v>45851</v>
       </c>
       <c r="C79" t="inlineStr">
@@ -7456,7 +7444,7 @@
     </row>
     <row r="80">
       <c r="A80" t="inlineStr"/>
-      <c r="B80" s="2" t="n">
+      <c r="B80" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C80" t="inlineStr">
@@ -7528,7 +7516,7 @@
     </row>
     <row r="81">
       <c r="A81" t="inlineStr"/>
-      <c r="B81" s="2" t="n">
+      <c r="B81" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C81" t="inlineStr">
@@ -7600,7 +7588,7 @@
     </row>
     <row r="82">
       <c r="A82" t="inlineStr"/>
-      <c r="B82" s="2" t="n">
+      <c r="B82" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C82" t="inlineStr">
@@ -7686,7 +7674,7 @@
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
-      <c r="B83" s="2" t="n">
+      <c r="B83" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C83" t="inlineStr">
@@ -7754,7 +7742,7 @@
     </row>
     <row r="84">
       <c r="A84" t="inlineStr"/>
-      <c r="B84" s="2" t="n">
+      <c r="B84" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C84" t="inlineStr">
@@ -7848,7 +7836,7 @@
     </row>
     <row r="85">
       <c r="A85" t="inlineStr"/>
-      <c r="B85" s="2" t="n">
+      <c r="B85" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C85" t="inlineStr">
@@ -7926,7 +7914,7 @@
     </row>
     <row r="86">
       <c r="A86" t="inlineStr"/>
-      <c r="B86" s="2" t="n">
+      <c r="B86" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C86" t="inlineStr">
@@ -8004,7 +7992,7 @@
     </row>
     <row r="87">
       <c r="A87" t="inlineStr"/>
-      <c r="B87" s="2" t="n">
+      <c r="B87" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C87" t="inlineStr">
@@ -8074,7 +8062,7 @@
     </row>
     <row r="88">
       <c r="A88" t="inlineStr"/>
-      <c r="B88" s="2" t="n">
+      <c r="B88" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C88" t="inlineStr">
@@ -8150,7 +8138,7 @@
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
-      <c r="B89" s="2" t="n">
+      <c r="B89" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C89" t="inlineStr">
@@ -8240,7 +8228,7 @@
     </row>
     <row r="90">
       <c r="A90" t="inlineStr"/>
-      <c r="B90" s="2" t="n">
+      <c r="B90" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C90" t="inlineStr">
@@ -8330,7 +8318,7 @@
     </row>
     <row r="91">
       <c r="A91" t="inlineStr"/>
-      <c r="B91" s="2" t="n">
+      <c r="B91" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C91" t="inlineStr">
@@ -8424,7 +8412,7 @@
     </row>
     <row r="92">
       <c r="A92" t="inlineStr"/>
-      <c r="B92" s="2" t="n">
+      <c r="B92" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C92" t="inlineStr">
@@ -8504,7 +8492,7 @@
     </row>
     <row r="93">
       <c r="A93" t="inlineStr"/>
-      <c r="B93" s="2" t="n">
+      <c r="B93" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C93" t="inlineStr">
@@ -8594,7 +8582,7 @@
     </row>
     <row r="94">
       <c r="A94" t="inlineStr"/>
-      <c r="B94" s="2" t="n">
+      <c r="B94" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C94" t="inlineStr">
@@ -8680,7 +8668,7 @@
     </row>
     <row r="95">
       <c r="A95" t="inlineStr"/>
-      <c r="B95" s="2" t="n">
+      <c r="B95" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C95" t="inlineStr">
@@ -8764,7 +8752,7 @@
     </row>
     <row r="96">
       <c r="A96" t="inlineStr"/>
-      <c r="B96" s="2" t="n">
+      <c r="B96" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C96" t="inlineStr">
@@ -8854,7 +8842,7 @@
     </row>
     <row r="97">
       <c r="A97" t="inlineStr"/>
-      <c r="B97" s="2" t="n">
+      <c r="B97" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C97" t="inlineStr">
@@ -8944,7 +8932,7 @@
     </row>
     <row r="98">
       <c r="A98" t="inlineStr"/>
-      <c r="B98" s="2" t="n">
+      <c r="B98" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C98" t="inlineStr">
@@ -9034,7 +9022,7 @@
     </row>
     <row r="99">
       <c r="A99" t="inlineStr"/>
-      <c r="B99" s="2" t="n">
+      <c r="B99" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C99" t="inlineStr">
@@ -9126,7 +9114,7 @@
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
-      <c r="B100" s="2" t="n">
+      <c r="B100" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C100" t="inlineStr">
@@ -9216,7 +9204,7 @@
     </row>
     <row r="101">
       <c r="A101" t="inlineStr"/>
-      <c r="B101" s="2" t="n">
+      <c r="B101" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C101" t="inlineStr">
@@ -9306,7 +9294,7 @@
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
-      <c r="B102" s="2" t="n">
+      <c r="B102" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C102" t="inlineStr">
@@ -9396,7 +9384,7 @@
     </row>
     <row r="103">
       <c r="A103" t="inlineStr"/>
-      <c r="B103" s="2" t="n">
+      <c r="B103" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C103" t="inlineStr">
@@ -9482,7 +9470,7 @@
     </row>
     <row r="104">
       <c r="A104" t="inlineStr"/>
-      <c r="B104" s="2" t="n">
+      <c r="B104" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C104" t="inlineStr">
@@ -9570,7 +9558,7 @@
     </row>
     <row r="105">
       <c r="A105" t="inlineStr"/>
-      <c r="B105" s="2" t="n">
+      <c r="B105" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C105" t="inlineStr">
@@ -9658,7 +9646,7 @@
     </row>
     <row r="106">
       <c r="A106" t="inlineStr"/>
-      <c r="B106" s="2" t="n">
+      <c r="B106" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C106" t="inlineStr">
@@ -9756,7 +9744,7 @@
     </row>
     <row r="107">
       <c r="A107" t="inlineStr"/>
-      <c r="B107" s="2" t="n">
+      <c r="B107" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C107" t="inlineStr">
@@ -9850,7 +9838,7 @@
     </row>
     <row r="108">
       <c r="A108" t="inlineStr"/>
-      <c r="B108" s="2" t="n">
+      <c r="B108" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C108" t="inlineStr">
@@ -9948,7 +9936,7 @@
     </row>
     <row r="109">
       <c r="A109" t="inlineStr"/>
-      <c r="B109" s="2" t="n">
+      <c r="B109" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C109" t="inlineStr">
@@ -10036,7 +10024,7 @@
     </row>
     <row r="110">
       <c r="A110" t="inlineStr"/>
-      <c r="B110" s="2" t="n">
+      <c r="B110" s="1" t="n">
         <v>45863</v>
       </c>
       <c r="C110" t="inlineStr">
@@ -10118,7 +10106,7 @@
     </row>
     <row r="111">
       <c r="A111" t="inlineStr"/>
-      <c r="B111" s="2" t="n">
+      <c r="B111" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C111" t="inlineStr">
@@ -10210,7 +10198,7 @@
     </row>
     <row r="112">
       <c r="A112" t="inlineStr"/>
-      <c r="B112" s="2" t="n">
+      <c r="B112" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C112" t="inlineStr">
@@ -10312,7 +10300,7 @@
     </row>
     <row r="113">
       <c r="A113" t="inlineStr"/>
-      <c r="B113" s="2" t="n">
+      <c r="B113" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C113" t="inlineStr">
@@ -10406,7 +10394,7 @@
     </row>
     <row r="114">
       <c r="A114" t="inlineStr"/>
-      <c r="B114" s="2" t="n">
+      <c r="B114" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C114" t="inlineStr">
@@ -10500,7 +10488,7 @@
     </row>
     <row r="115">
       <c r="A115" t="inlineStr"/>
-      <c r="B115" s="2" t="n">
+      <c r="B115" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C115" t="inlineStr">
@@ -10594,7 +10582,7 @@
     </row>
     <row r="116">
       <c r="A116" t="inlineStr"/>
-      <c r="B116" s="2" t="n">
+      <c r="B116" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C116" t="inlineStr">
@@ -10688,7 +10676,7 @@
     </row>
     <row r="117">
       <c r="A117" t="inlineStr"/>
-      <c r="B117" s="2" t="n">
+      <c r="B117" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C117" t="inlineStr">
@@ -10778,7 +10766,7 @@
     </row>
     <row r="118">
       <c r="A118" t="inlineStr"/>
-      <c r="B118" s="2" t="n">
+      <c r="B118" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C118" t="inlineStr">
@@ -10872,7 +10860,7 @@
     </row>
     <row r="119">
       <c r="A119" t="inlineStr"/>
-      <c r="B119" s="2" t="n">
+      <c r="B119" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C119" t="inlineStr">
@@ -10962,7 +10950,7 @@
     </row>
     <row r="120">
       <c r="A120" t="inlineStr"/>
-      <c r="B120" s="2" t="n">
+      <c r="B120" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C120" t="inlineStr">
@@ -11052,7 +11040,7 @@
     </row>
     <row r="121">
       <c r="A121" t="inlineStr"/>
-      <c r="B121" s="2" t="n">
+      <c r="B121" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C121" t="inlineStr">
@@ -11140,7 +11128,7 @@
     </row>
     <row r="122">
       <c r="A122" t="inlineStr"/>
-      <c r="B122" s="2" t="n">
+      <c r="B122" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C122" t="inlineStr">
@@ -11234,7 +11222,7 @@
     </row>
     <row r="123">
       <c r="A123" t="inlineStr"/>
-      <c r="B123" s="2" t="n">
+      <c r="B123" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C123" t="inlineStr">
@@ -11324,7 +11312,7 @@
     </row>
     <row r="124">
       <c r="A124" t="inlineStr"/>
-      <c r="B124" s="2" t="n">
+      <c r="B124" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C124" t="inlineStr">
@@ -11420,7 +11408,7 @@
     </row>
     <row r="125">
       <c r="A125" t="inlineStr"/>
-      <c r="B125" s="2" t="n">
+      <c r="B125" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C125" t="inlineStr">
@@ -11516,7 +11504,7 @@
     </row>
     <row r="126">
       <c r="A126" t="inlineStr"/>
-      <c r="B126" s="2" t="n">
+      <c r="B126" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C126" t="inlineStr">
@@ -11610,7 +11598,7 @@
     </row>
     <row r="127">
       <c r="A127" t="inlineStr"/>
-      <c r="B127" s="2" t="n">
+      <c r="B127" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C127" t="inlineStr">
@@ -11702,7 +11690,7 @@
     </row>
     <row r="128">
       <c r="A128" t="inlineStr"/>
-      <c r="B128" s="2" t="n">
+      <c r="B128" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C128" t="inlineStr">
@@ -11796,7 +11784,7 @@
     </row>
     <row r="129">
       <c r="A129" t="inlineStr"/>
-      <c r="B129" s="2" t="n">
+      <c r="B129" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C129" t="inlineStr">
@@ -11886,7 +11874,7 @@
     </row>
     <row r="130">
       <c r="A130" t="inlineStr"/>
-      <c r="B130" s="2" t="n">
+      <c r="B130" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C130" t="inlineStr">
@@ -11982,7 +11970,7 @@
     </row>
     <row r="131">
       <c r="A131" t="inlineStr"/>
-      <c r="B131" s="2" t="n">
+      <c r="B131" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C131" t="inlineStr">
@@ -12074,7 +12062,7 @@
     </row>
     <row r="132">
       <c r="A132" t="inlineStr"/>
-      <c r="B132" s="2" t="n">
+      <c r="B132" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C132" t="inlineStr">
@@ -12164,7 +12152,7 @@
     </row>
     <row r="133">
       <c r="A133" t="inlineStr"/>
-      <c r="B133" s="2" t="n">
+      <c r="B133" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C133" t="inlineStr">
@@ -12256,7 +12244,7 @@
     </row>
     <row r="134">
       <c r="A134" t="inlineStr"/>
-      <c r="B134" s="2" t="n">
+      <c r="B134" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C134" t="inlineStr">
@@ -12346,7 +12334,7 @@
     </row>
     <row r="135">
       <c r="A135" t="inlineStr"/>
-      <c r="B135" s="2" t="n">
+      <c r="B135" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C135" t="inlineStr">
@@ -12434,7 +12422,7 @@
     </row>
     <row r="136">
       <c r="A136" t="inlineStr"/>
-      <c r="B136" s="2" t="n">
+      <c r="B136" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C136" t="inlineStr">
@@ -12508,7 +12496,7 @@
     </row>
     <row r="137">
       <c r="A137" t="inlineStr"/>
-      <c r="B137" s="2" t="n">
+      <c r="B137" s="1" t="n">
         <v>45864</v>
       </c>
       <c r="C137" t="inlineStr">
@@ -12588,7 +12576,7 @@
     </row>
     <row r="138">
       <c r="A138" t="inlineStr"/>
-      <c r="B138" s="2" t="n">
+      <c r="B138" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="C138" t="inlineStr">
@@ -12668,7 +12656,7 @@
     </row>
     <row r="139">
       <c r="A139" t="inlineStr"/>
-      <c r="B139" s="2" t="n">
+      <c r="B139" s="1" t="n">
         <v>45875</v>
       </c>
       <c r="C139" t="inlineStr">
@@ -12774,7 +12762,7 @@
     </row>
     <row r="140">
       <c r="A140" t="inlineStr"/>
-      <c r="B140" s="2" t="n">
+      <c r="B140" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="C140" t="inlineStr">
@@ -12862,7 +12850,7 @@
     </row>
     <row r="141">
       <c r="A141" t="inlineStr"/>
-      <c r="B141" s="2" t="n">
+      <c r="B141" s="1" t="n">
         <v>45933</v>
       </c>
       <c r="C141" t="inlineStr">
@@ -12926,7 +12914,7 @@
     </row>
     <row r="142">
       <c r="A142" t="inlineStr"/>
-      <c r="B142" s="2" t="n">
+      <c r="B142" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="C142" t="inlineStr">
@@ -12988,7 +12976,7 @@
     </row>
     <row r="143">
       <c r="A143" t="inlineStr"/>
-      <c r="B143" s="2" t="n">
+      <c r="B143" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="C143" t="inlineStr">
@@ -13058,7 +13046,7 @@
     </row>
     <row r="144">
       <c r="A144" t="inlineStr"/>
-      <c r="B144" s="2" t="n">
+      <c r="B144" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="C144" t="inlineStr">
@@ -15040,6 +15028,94 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>CRRT</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026-05-21 21:11:49</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr"/>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>E3B0C442</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="inlineStr"/>
+      <c r="L164" t="inlineStr"/>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr"/>
+      <c r="P164" t="inlineStr"/>
+      <c r="Q164" t="inlineStr"/>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="S164" t="inlineStr"/>
+      <c r="T164" t="inlineStr"/>
+      <c r="U164" t="inlineStr"/>
+      <c r="V164" t="inlineStr"/>
+      <c r="W164" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="X164" t="inlineStr"/>
+      <c r="Y164" t="inlineStr"/>
+      <c r="Z164" t="inlineStr"/>
+      <c r="AA164" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="AB164" t="inlineStr"/>
+      <c r="AC164" t="inlineStr"/>
+      <c r="AD164" t="inlineStr"/>
+      <c r="AE164" t="inlineStr"/>
+      <c r="AF164" t="inlineStr">
+        <is>
+          <t>Tidak Diketahui</t>
+        </is>
+      </c>
+      <c r="AG164" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AH164" t="inlineStr">
+        <is>
+          <t>Non-Survivor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>